<commit_message>
ref: refactored export as PDF PO
</commit_message>
<xml_diff>
--- a/procurement_documents/PO Template.xlsx
+++ b/procurement_documents/PO Template.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73FF062A-9C2E-4060-A0BE-97F28908FB60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70871D63-A8BA-4174-B2A6-CFD010F39A83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{1AFC0673-2000-41F1-BB87-1A913DCADB25}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{1AFC0673-2000-41F1-BB87-1A913DCADB25}"/>
   </bookViews>
   <sheets>
     <sheet name="PO" sheetId="1" r:id="rId1"/>
     <sheet name="PO with Mapping" sheetId="4" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">PO!$A$1:$F$55</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">PO!$A$1:$F$56</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'PO with Mapping'!$A$1:$F$55</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="63">
   <si>
     <t>Stock/Property No.</t>
   </si>
@@ -254,13 +254,16 @@
   </si>
   <si>
     <t>user-&gt;role_name where user-&gt;role_id = 68</t>
+  </si>
+  <si>
+    <t>po_date_delivery</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -343,6 +346,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -352,7 +362,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="43">
+  <borders count="44">
     <border>
       <left/>
       <right/>
@@ -858,11 +868,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -958,6 +979,30 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -967,31 +1012,34 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1000,10 +1048,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1035,59 +1105,68 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1488,87 +1567,87 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25838C5E-5DCD-4782-8BB2-08A0BAFE6B1C}">
-  <sheetPr>
+  <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="10.7109375" customWidth="1"/>
-    <col min="3" max="3" width="50.7109375" customWidth="1"/>
-    <col min="4" max="6" width="10.7109375" customWidth="1"/>
+    <col min="1" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="55.7109375" customWidth="1"/>
+    <col min="4" max="6" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="51" t="e" vm="1">
+      <c r="A1" s="80" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="63" t="s">
+      <c r="B1" s="82" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="64"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="66" t="s">
+      <c r="C1" s="83"/>
+      <c r="D1" s="84"/>
+      <c r="E1" s="85" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="67"/>
+      <c r="F1" s="86"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="52"/>
-      <c r="B2" s="68" t="s">
+      <c r="A2" s="81"/>
+      <c r="B2" s="87" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="70" t="s">
+      <c r="C2" s="87"/>
+      <c r="D2" s="88"/>
+      <c r="E2" s="89" t="s">
         <v>36</v>
       </c>
-      <c r="F2" s="71"/>
+      <c r="F2" s="90"/>
     </row>
     <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="72" t="s">
+      <c r="A4" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="73"/>
-      <c r="C4" s="61"/>
-      <c r="D4" s="62"/>
+      <c r="B4" s="99"/>
+      <c r="C4" s="95"/>
+      <c r="D4" s="94"/>
       <c r="E4" s="22" t="s">
         <v>18</v>
       </c>
       <c r="F4" s="33"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="74" t="s">
+      <c r="A5" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="53"/>
-      <c r="D5" s="54"/>
+      <c r="B5" s="100"/>
+      <c r="C5" s="96"/>
+      <c r="D5" s="75"/>
       <c r="E5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="F5" s="34"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="74" t="s">
+      <c r="A6" s="63" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="53"/>
-      <c r="D6" s="54"/>
+      <c r="B6" s="100"/>
+      <c r="C6" s="96"/>
+      <c r="D6" s="75"/>
       <c r="E6" s="25" t="s">
         <v>20</v>
       </c>
       <c r="F6" s="34"/>
     </row>
     <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="76" t="s">
+      <c r="A7" s="66" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="77"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="56"/>
+      <c r="B7" s="101"/>
+      <c r="C7" s="97"/>
+      <c r="D7" s="79"/>
       <c r="E7" s="24" t="s">
         <v>21</v>
       </c>
@@ -1587,33 +1666,33 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="11"/>
-      <c r="B9" s="50" t="s">
+      <c r="B9" s="114" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="50"/>
-      <c r="D9" s="50"/>
-      <c r="E9" s="50"/>
+      <c r="C9" s="114"/>
+      <c r="D9" s="114"/>
+      <c r="E9" s="114"/>
       <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="78" t="s">
+      <c r="A10" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="58"/>
-      <c r="C10" s="57"/>
-      <c r="D10" s="58"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="102"/>
+      <c r="D10" s="103"/>
       <c r="E10" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F10" s="36"/>
     </row>
     <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="79" t="s">
+      <c r="A11" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="80"/>
-      <c r="C11" s="59"/>
-      <c r="D11" s="60"/>
+      <c r="B11" s="67"/>
+      <c r="C11" s="68"/>
+      <c r="D11" s="69"/>
       <c r="E11" s="40" t="s">
         <v>23</v>
       </c>
@@ -1644,227 +1723,227 @@
       <c r="B13" s="1"/>
       <c r="C13" s="3"/>
       <c r="D13" s="1"/>
-      <c r="E13" s="81"/>
-      <c r="F13" s="82"/>
+      <c r="E13" s="47"/>
+      <c r="F13" s="48"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="35"/>
       <c r="B14" s="1"/>
       <c r="C14" s="3"/>
       <c r="D14" s="1"/>
-      <c r="E14" s="83"/>
-      <c r="F14" s="82"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="48"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="35"/>
       <c r="B15" s="1"/>
       <c r="C15" s="3"/>
       <c r="D15" s="1"/>
-      <c r="E15" s="81"/>
-      <c r="F15" s="82"/>
+      <c r="E15" s="47"/>
+      <c r="F15" s="48"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="35"/>
       <c r="B16" s="1"/>
       <c r="C16" s="3"/>
       <c r="D16" s="1"/>
-      <c r="E16" s="81"/>
-      <c r="F16" s="82"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="48"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="35"/>
       <c r="B17" s="1"/>
       <c r="C17" s="3"/>
       <c r="D17" s="1"/>
-      <c r="E17" s="81"/>
-      <c r="F17" s="82"/>
+      <c r="E17" s="47"/>
+      <c r="F17" s="48"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="35"/>
       <c r="B18" s="1"/>
       <c r="C18" s="3"/>
       <c r="D18" s="1"/>
-      <c r="E18" s="81"/>
-      <c r="F18" s="82"/>
+      <c r="E18" s="47"/>
+      <c r="F18" s="48"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="35"/>
       <c r="B19" s="1"/>
       <c r="C19" s="3"/>
       <c r="D19" s="1"/>
-      <c r="E19" s="81"/>
-      <c r="F19" s="82"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="48"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="35"/>
       <c r="B20" s="1"/>
       <c r="C20" s="3"/>
       <c r="D20" s="1"/>
-      <c r="E20" s="81"/>
-      <c r="F20" s="82"/>
+      <c r="E20" s="47"/>
+      <c r="F20" s="48"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="35"/>
       <c r="B21" s="1"/>
       <c r="C21" s="3"/>
       <c r="D21" s="1"/>
-      <c r="E21" s="81"/>
-      <c r="F21" s="82"/>
+      <c r="E21" s="47"/>
+      <c r="F21" s="48"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="35"/>
       <c r="B22" s="1"/>
       <c r="C22" s="3"/>
       <c r="D22" s="1"/>
-      <c r="E22" s="81"/>
-      <c r="F22" s="82"/>
+      <c r="E22" s="47"/>
+      <c r="F22" s="48"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="35"/>
       <c r="B23" s="1"/>
       <c r="C23" s="3"/>
       <c r="D23" s="1"/>
-      <c r="E23" s="81"/>
-      <c r="F23" s="82"/>
+      <c r="E23" s="47"/>
+      <c r="F23" s="48"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="35"/>
       <c r="B24" s="1"/>
       <c r="C24" s="3"/>
       <c r="D24" s="1"/>
-      <c r="E24" s="81"/>
-      <c r="F24" s="82"/>
+      <c r="E24" s="47"/>
+      <c r="F24" s="48"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="35"/>
       <c r="B25" s="1"/>
       <c r="C25" s="3"/>
       <c r="D25" s="1"/>
-      <c r="E25" s="81"/>
-      <c r="F25" s="82"/>
+      <c r="E25" s="47"/>
+      <c r="F25" s="48"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="35"/>
       <c r="B26" s="1"/>
       <c r="C26" s="3"/>
       <c r="D26" s="1"/>
-      <c r="E26" s="81"/>
-      <c r="F26" s="82"/>
+      <c r="E26" s="47"/>
+      <c r="F26" s="48"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="35"/>
       <c r="B27" s="1"/>
       <c r="C27" s="3"/>
       <c r="D27" s="1"/>
-      <c r="E27" s="81"/>
-      <c r="F27" s="82"/>
+      <c r="E27" s="47"/>
+      <c r="F27" s="48"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="35"/>
       <c r="B28" s="1"/>
       <c r="C28" s="3"/>
       <c r="D28" s="1"/>
-      <c r="E28" s="81"/>
-      <c r="F28" s="82"/>
+      <c r="E28" s="47"/>
+      <c r="F28" s="48"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="35"/>
       <c r="B29" s="1"/>
       <c r="C29" s="3"/>
       <c r="D29" s="1"/>
-      <c r="E29" s="81"/>
-      <c r="F29" s="82"/>
+      <c r="E29" s="47"/>
+      <c r="F29" s="48"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="35"/>
       <c r="B30" s="1"/>
       <c r="C30" s="3"/>
       <c r="D30" s="1"/>
-      <c r="E30" s="81"/>
-      <c r="F30" s="82"/>
+      <c r="E30" s="47"/>
+      <c r="F30" s="48"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="35"/>
       <c r="B31" s="1"/>
       <c r="C31" s="3"/>
       <c r="D31" s="1"/>
-      <c r="E31" s="81"/>
-      <c r="F31" s="82"/>
+      <c r="E31" s="47"/>
+      <c r="F31" s="48"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="35"/>
       <c r="B32" s="1"/>
       <c r="C32" s="3"/>
       <c r="D32" s="1"/>
-      <c r="E32" s="81"/>
-      <c r="F32" s="82"/>
+      <c r="E32" s="47"/>
+      <c r="F32" s="48"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="35"/>
       <c r="B33" s="1"/>
       <c r="C33" s="3"/>
       <c r="D33" s="1"/>
-      <c r="E33" s="81"/>
-      <c r="F33" s="82"/>
+      <c r="E33" s="47"/>
+      <c r="F33" s="48"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="35"/>
       <c r="B34" s="1"/>
       <c r="C34" s="3"/>
       <c r="D34" s="1"/>
-      <c r="E34" s="81"/>
-      <c r="F34" s="82"/>
+      <c r="E34" s="47"/>
+      <c r="F34" s="48"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="35"/>
       <c r="B35" s="1"/>
       <c r="C35" s="3"/>
       <c r="D35" s="1"/>
-      <c r="E35" s="81"/>
-      <c r="F35" s="82"/>
+      <c r="E35" s="47"/>
+      <c r="F35" s="48"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="35"/>
       <c r="B36" s="1"/>
       <c r="C36" s="3"/>
       <c r="D36" s="1"/>
-      <c r="E36" s="81"/>
-      <c r="F36" s="82"/>
+      <c r="E36" s="47"/>
+      <c r="F36" s="48"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="35"/>
       <c r="B37" s="1"/>
       <c r="C37" s="3"/>
       <c r="D37" s="1"/>
-      <c r="E37" s="81"/>
-      <c r="F37" s="82"/>
+      <c r="E37" s="47"/>
+      <c r="F37" s="48"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="86"/>
-      <c r="B38" s="84"/>
-      <c r="C38" s="84"/>
-      <c r="D38" s="84"/>
-      <c r="E38" s="84"/>
-      <c r="F38" s="85"/>
+      <c r="A38" s="104"/>
+      <c r="B38" s="105"/>
+      <c r="C38" s="105"/>
+      <c r="D38" s="105"/>
+      <c r="E38" s="105"/>
+      <c r="F38" s="50"/>
     </row>
     <row r="39" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="90"/>
-      <c r="B39" s="89"/>
-      <c r="C39" s="89"/>
-      <c r="D39" s="89"/>
-      <c r="E39" s="91"/>
-      <c r="F39" s="41"/>
+      <c r="A39" s="106"/>
+      <c r="B39" s="107"/>
+      <c r="C39" s="107"/>
+      <c r="D39" s="107"/>
+      <c r="E39" s="108"/>
+      <c r="F39" s="109"/>
     </row>
     <row r="40" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="47" t="s">
+      <c r="A41" s="55" t="s">
         <v>38</v>
       </c>
-      <c r="B41" s="48"/>
-      <c r="C41" s="48"/>
-      <c r="D41" s="48"/>
-      <c r="E41" s="48"/>
-      <c r="F41" s="49"/>
+      <c r="B41" s="56"/>
+      <c r="C41" s="56"/>
+      <c r="D41" s="56"/>
+      <c r="E41" s="56"/>
+      <c r="F41" s="57"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="9"/>
@@ -1882,17 +1961,17 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="9"/>
-      <c r="D44" s="87"/>
-      <c r="E44" s="87"/>
-      <c r="F44" s="88"/>
+      <c r="D44" s="58"/>
+      <c r="E44" s="58"/>
+      <c r="F44" s="59"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="9"/>
       <c r="B45" s="6"/>
       <c r="C45" s="6"/>
-      <c r="D45" s="93"/>
-      <c r="E45" s="93"/>
-      <c r="F45" s="94"/>
+      <c r="D45" s="110"/>
+      <c r="E45" s="110"/>
+      <c r="F45" s="111"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="9"/>
@@ -1928,7 +2007,7 @@
       <c r="F50" s="12"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="23" t="s">
+      <c r="A51" s="112" t="s">
         <v>28</v>
       </c>
       <c r="B51" s="4" t="s">
@@ -1936,7 +2015,7 @@
       </c>
       <c r="C51" s="4"/>
       <c r="D51" s="5"/>
-      <c r="E51" s="38" t="s">
+      <c r="E51" s="113" t="s">
         <v>33</v>
       </c>
       <c r="F51" s="13" t="s">
@@ -1989,6 +2068,20 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="A6:B6"/>
     <mergeCell ref="D44:F44"/>
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A38:E38"/>
@@ -1998,30 +2091,16 @@
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A41:F41"/>
     <mergeCell ref="B9:E9"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A6:B6"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="93" fitToWidth="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="91" fitToWidth="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CD9717F-76FE-48EB-A301-8321B71100D8}">
-  <sheetPr>
+  <sheetPr codeName="Sheet2">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H56"/>
@@ -2033,41 +2112,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="51" t="e" vm="1">
+      <c r="A1" s="80" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="63" t="s">
+      <c r="B1" s="82" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="64"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="66" t="s">
+      <c r="C1" s="83"/>
+      <c r="D1" s="84"/>
+      <c r="E1" s="85" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="67"/>
+      <c r="F1" s="86"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="52"/>
-      <c r="B2" s="68" t="s">
+      <c r="A2" s="81"/>
+      <c r="B2" s="87" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="70" t="s">
+      <c r="C2" s="87"/>
+      <c r="D2" s="88"/>
+      <c r="E2" s="89" t="s">
         <v>36</v>
       </c>
-      <c r="F2" s="71"/>
+      <c r="F2" s="90"/>
     </row>
     <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="72" t="s">
+      <c r="A4" s="91" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="73"/>
-      <c r="C4" s="61" t="s">
+      <c r="B4" s="92"/>
+      <c r="C4" s="93" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="62"/>
+      <c r="D4" s="94"/>
       <c r="E4" s="22" t="s">
         <v>18</v>
       </c>
@@ -2076,14 +2155,14 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="74" t="s">
+      <c r="A5" s="72" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="53" t="s">
+      <c r="B5" s="73"/>
+      <c r="C5" s="74" t="s">
         <v>41</v>
       </c>
-      <c r="D5" s="54"/>
+      <c r="D5" s="75"/>
       <c r="E5" s="2" t="s">
         <v>19</v>
       </c>
@@ -2092,14 +2171,14 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="74" t="s">
+      <c r="A6" s="72" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="53" t="s">
+      <c r="B6" s="73"/>
+      <c r="C6" s="74" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="54"/>
+      <c r="D6" s="75"/>
       <c r="E6" s="25" t="s">
         <v>20</v>
       </c>
@@ -2112,10 +2191,10 @@
         <v>13</v>
       </c>
       <c r="B7" s="77"/>
-      <c r="C7" s="55" t="s">
+      <c r="C7" s="78" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="56"/>
+      <c r="D7" s="79"/>
       <c r="E7" s="24" t="s">
         <v>21</v>
       </c>
@@ -2136,23 +2215,23 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="11"/>
-      <c r="B9" s="50" t="s">
+      <c r="B9" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="50"/>
-      <c r="D9" s="50"/>
-      <c r="E9" s="50"/>
+      <c r="C9" s="62"/>
+      <c r="D9" s="62"/>
+      <c r="E9" s="62"/>
       <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="78" t="s">
+      <c r="A10" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="58"/>
-      <c r="C10" s="57" t="s">
+      <c r="B10" s="64"/>
+      <c r="C10" s="65" t="s">
         <v>48</v>
       </c>
-      <c r="D10" s="58"/>
+      <c r="D10" s="64"/>
       <c r="E10" s="39" t="s">
         <v>22</v>
       </c>
@@ -2161,14 +2240,14 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="79" t="s">
+      <c r="A11" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="80"/>
-      <c r="C11" s="59" t="s">
-        <v>49</v>
-      </c>
-      <c r="D11" s="60"/>
+      <c r="B11" s="67"/>
+      <c r="C11" s="68" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" s="69"/>
       <c r="E11" s="40" t="s">
         <v>23</v>
       </c>
@@ -2209,10 +2288,10 @@
       <c r="D13" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E13" s="81" t="s">
+      <c r="E13" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="F13" s="82" t="s">
+      <c r="F13" s="48" t="s">
         <v>58</v>
       </c>
     </row>
@@ -2221,225 +2300,225 @@
       <c r="B14" s="1"/>
       <c r="C14" s="3"/>
       <c r="D14" s="1"/>
-      <c r="E14" s="83"/>
-      <c r="F14" s="82"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="48"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="35"/>
       <c r="B15" s="1"/>
       <c r="C15" s="3"/>
       <c r="D15" s="1"/>
-      <c r="E15" s="81"/>
-      <c r="F15" s="82"/>
+      <c r="E15" s="47"/>
+      <c r="F15" s="48"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="35"/>
       <c r="B16" s="1"/>
       <c r="C16" s="3"/>
       <c r="D16" s="1"/>
-      <c r="E16" s="81"/>
-      <c r="F16" s="82"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="48"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="35"/>
       <c r="B17" s="1"/>
       <c r="C17" s="3"/>
       <c r="D17" s="1"/>
-      <c r="E17" s="81"/>
-      <c r="F17" s="82"/>
+      <c r="E17" s="47"/>
+      <c r="F17" s="48"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="35"/>
       <c r="B18" s="1"/>
       <c r="C18" s="3"/>
       <c r="D18" s="1"/>
-      <c r="E18" s="81"/>
-      <c r="F18" s="82"/>
+      <c r="E18" s="47"/>
+      <c r="F18" s="48"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="35"/>
       <c r="B19" s="1"/>
       <c r="C19" s="3"/>
       <c r="D19" s="1"/>
-      <c r="E19" s="81"/>
-      <c r="F19" s="82"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="48"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="35"/>
       <c r="B20" s="1"/>
       <c r="C20" s="3"/>
       <c r="D20" s="1"/>
-      <c r="E20" s="81"/>
-      <c r="F20" s="82"/>
+      <c r="E20" s="47"/>
+      <c r="F20" s="48"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="35"/>
       <c r="B21" s="1"/>
       <c r="C21" s="3"/>
       <c r="D21" s="1"/>
-      <c r="E21" s="81"/>
-      <c r="F21" s="82"/>
+      <c r="E21" s="47"/>
+      <c r="F21" s="48"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="35"/>
       <c r="B22" s="1"/>
       <c r="C22" s="3"/>
       <c r="D22" s="1"/>
-      <c r="E22" s="81"/>
-      <c r="F22" s="82"/>
+      <c r="E22" s="47"/>
+      <c r="F22" s="48"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="35"/>
       <c r="B23" s="1"/>
       <c r="C23" s="3"/>
       <c r="D23" s="1"/>
-      <c r="E23" s="81"/>
-      <c r="F23" s="82"/>
+      <c r="E23" s="47"/>
+      <c r="F23" s="48"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="35"/>
       <c r="B24" s="1"/>
       <c r="C24" s="3"/>
       <c r="D24" s="1"/>
-      <c r="E24" s="81"/>
-      <c r="F24" s="82"/>
+      <c r="E24" s="47"/>
+      <c r="F24" s="48"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="35"/>
       <c r="B25" s="1"/>
       <c r="C25" s="3"/>
       <c r="D25" s="1"/>
-      <c r="E25" s="81"/>
-      <c r="F25" s="82"/>
+      <c r="E25" s="47"/>
+      <c r="F25" s="48"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="35"/>
       <c r="B26" s="1"/>
       <c r="C26" s="3"/>
       <c r="D26" s="1"/>
-      <c r="E26" s="81"/>
-      <c r="F26" s="82"/>
+      <c r="E26" s="47"/>
+      <c r="F26" s="48"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="35"/>
       <c r="B27" s="1"/>
       <c r="C27" s="3"/>
       <c r="D27" s="1"/>
-      <c r="E27" s="81"/>
-      <c r="F27" s="82"/>
+      <c r="E27" s="47"/>
+      <c r="F27" s="48"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="35"/>
       <c r="B28" s="1"/>
       <c r="C28" s="3"/>
       <c r="D28" s="1"/>
-      <c r="E28" s="81"/>
-      <c r="F28" s="82"/>
+      <c r="E28" s="47"/>
+      <c r="F28" s="48"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="35"/>
       <c r="B29" s="1"/>
       <c r="C29" s="3"/>
       <c r="D29" s="1"/>
-      <c r="E29" s="81"/>
-      <c r="F29" s="82"/>
+      <c r="E29" s="47"/>
+      <c r="F29" s="48"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="35"/>
       <c r="B30" s="1"/>
       <c r="C30" s="3"/>
       <c r="D30" s="1"/>
-      <c r="E30" s="81"/>
-      <c r="F30" s="82"/>
+      <c r="E30" s="47"/>
+      <c r="F30" s="48"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="35"/>
       <c r="B31" s="1"/>
       <c r="C31" s="3"/>
       <c r="D31" s="1"/>
-      <c r="E31" s="81"/>
-      <c r="F31" s="82"/>
+      <c r="E31" s="47"/>
+      <c r="F31" s="48"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="35"/>
       <c r="B32" s="1"/>
       <c r="C32" s="3"/>
       <c r="D32" s="1"/>
-      <c r="E32" s="81"/>
-      <c r="F32" s="82"/>
+      <c r="E32" s="47"/>
+      <c r="F32" s="48"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="35"/>
       <c r="B33" s="1"/>
       <c r="C33" s="3"/>
       <c r="D33" s="1"/>
-      <c r="E33" s="81"/>
-      <c r="F33" s="82"/>
+      <c r="E33" s="47"/>
+      <c r="F33" s="48"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="35"/>
       <c r="B34" s="1"/>
       <c r="C34" s="3"/>
       <c r="D34" s="1"/>
-      <c r="E34" s="81"/>
-      <c r="F34" s="82"/>
+      <c r="E34" s="47"/>
+      <c r="F34" s="48"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="35"/>
       <c r="B35" s="1"/>
       <c r="C35" s="3"/>
       <c r="D35" s="1"/>
-      <c r="E35" s="81"/>
-      <c r="F35" s="82"/>
+      <c r="E35" s="47"/>
+      <c r="F35" s="48"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="35"/>
       <c r="B36" s="1"/>
       <c r="C36" s="3"/>
       <c r="D36" s="1"/>
-      <c r="E36" s="81"/>
-      <c r="F36" s="82"/>
+      <c r="E36" s="47"/>
+      <c r="F36" s="48"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="35"/>
       <c r="B37" s="1"/>
       <c r="C37" s="3"/>
       <c r="D37" s="1"/>
-      <c r="E37" s="81"/>
-      <c r="F37" s="82"/>
+      <c r="E37" s="47"/>
+      <c r="F37" s="48"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="86" t="s">
+      <c r="A38" s="70" t="s">
         <v>55</v>
       </c>
-      <c r="B38" s="84"/>
-      <c r="C38" s="84"/>
-      <c r="D38" s="84"/>
-      <c r="E38" s="84"/>
-      <c r="F38" s="85"/>
+      <c r="B38" s="71"/>
+      <c r="C38" s="71"/>
+      <c r="D38" s="71"/>
+      <c r="E38" s="71"/>
+      <c r="F38" s="50"/>
     </row>
     <row r="39" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="90" t="s">
+      <c r="A39" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="B39" s="89"/>
-      <c r="C39" s="89"/>
-      <c r="D39" s="89"/>
-      <c r="E39" s="91"/>
+      <c r="B39" s="53"/>
+      <c r="C39" s="53"/>
+      <c r="D39" s="53"/>
+      <c r="E39" s="54"/>
       <c r="F39" s="41" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="47" t="s">
+      <c r="A41" s="55" t="s">
         <v>38</v>
       </c>
-      <c r="B41" s="48"/>
-      <c r="C41" s="48"/>
-      <c r="D41" s="48"/>
-      <c r="E41" s="48"/>
-      <c r="F41" s="49"/>
+      <c r="B41" s="56"/>
+      <c r="C41" s="56"/>
+      <c r="D41" s="56"/>
+      <c r="E41" s="56"/>
+      <c r="F41" s="57"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="9"/>
@@ -2457,21 +2536,21 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="9"/>
-      <c r="D44" s="87" t="s">
+      <c r="D44" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="E44" s="87"/>
-      <c r="F44" s="88"/>
+      <c r="E44" s="58"/>
+      <c r="F44" s="59"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="9"/>
       <c r="B45" s="6"/>
       <c r="C45" s="6"/>
-      <c r="D45" s="93" t="s">
+      <c r="D45" s="60" t="s">
         <v>61</v>
       </c>
-      <c r="E45" s="93"/>
-      <c r="F45" s="94"/>
+      <c r="E45" s="60"/>
+      <c r="F45" s="61"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="9"/>
@@ -2567,12 +2646,25 @@
       <c r="F55" s="18"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F56" s="92" t="s">
+      <c r="F56" s="51" t="s">
         <v>56</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A41:F41"/>
     <mergeCell ref="D44:F44"/>
@@ -2583,19 +2675,6 @@
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:D4"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>